<commit_message>
map-excel: title-hygiene fix per LEAD spot-check — annotations/slugs never in title cells, team-facing language
- Review D14: slug+annotation title replaced with the e-com sheet exact product
  title (Jivo Extra Light Olive Oil - 3 Litre …); slug moved to the id column,
  annotation to the reason column
- blessed -> owner-verified in all evidence/consensus/reason/note text (MRP
  integrity F2/F4/F6 + anywhere else, team-facing)
- former ⚠ title markers moved out of title cells into the note column (title
  blank when no on-page title exists); unpriced col1 shows (title not captured)
- new post-write assert_title_hygiene: 0 slug-shaped titles, 0 banned
  annotations in any title cell, 0 blessed jargon workbook-wide — fails loudly
- invariants re-asserted: 286/286 price cells hyperlinked, 0 no-link
</commit_message>
<xml_diff>
--- a/tools/pricematch/Jivo-SKU-Master-Map-2026-06-06.xlsx
+++ b/tools/pricematch/Jivo-SKU-Master-Map-2026-06-06.xlsx
@@ -5566,7 +5566,7 @@
       </c>
       <c r="M27" s="7" t="inlineStr">
         <is>
-          <t>identity verified (v2 CORRECT); prid owner-blessed from master sheet BLINKIT URL</t>
+          <t>identity verified (v2 CORRECT); prid owner-verified from master sheet BLINKIT URL</t>
         </is>
       </c>
     </row>
@@ -5890,7 +5890,7 @@
       </c>
       <c r="M33" s="7" t="inlineStr">
         <is>
-          <t>blessed pid is a 'pack 3 - 1 litre each' listing (owner counts 3x1L as the 3L SKU). Unpriced today.</t>
+          <t>owner-verified pid is a 'pack 3 - 1 litre each' listing (owner counts 3x1L as the 3L SKU). Unpriced today.</t>
         </is>
       </c>
     </row>
@@ -6273,7 +6273,7 @@
       </c>
       <c r="M40" s="7" t="inlineStr">
         <is>
-          <t>identity verified (v2 CORRECT); prid owner-blessed from master sheet BLINKIT URL</t>
+          <t>identity verified (v2 CORRECT); prid owner-verified from master sheet BLINKIT URL</t>
         </is>
       </c>
     </row>
@@ -7278,7 +7278,7 @@
       </c>
       <c r="M59" s="7" t="inlineStr">
         <is>
-          <t>mrp 398 on both fk listings; amazon+amazon-fresh show 399 (Re.1 rounding) vs master 695 -&gt; master_mrp_stale per LEAD ruling; identity owner-blessed.</t>
+          <t>mrp 398 on both fk listings; amazon+amazon-fresh show 399 (Re.1 rounding) vs master 695 -&gt; master_mrp_stale per LEAD ruling; identity owner-verified.</t>
         </is>
       </c>
     </row>
@@ -7916,7 +7916,7 @@
       </c>
       <c r="M71" s="7" t="inlineStr">
         <is>
-          <t>identity verified (v2 CORRECT); prid owner-blessed from master sheet BLINKIT URL</t>
+          <t>identity verified (v2 CORRECT); prid owner-verified from master sheet BLINKIT URL</t>
         </is>
       </c>
     </row>
@@ -8195,7 +8195,7 @@
       </c>
       <c r="M76" s="7" t="inlineStr">
         <is>
-          <t>blessed pid is the 1+1L PET pack @ mrp 2998 (= 2 x 1499 EL-1L master); the single 2L-can listing EDOGHZTJZEYQJGME also shows 2998 and zepto shows 2998 x34, while fresh/now/blinkit/bigbasket show master 2799 -&gt; mixed pack-variant pricing, flagged in master_mrp_stale with caveat.</t>
+          <t>owner-verified pid is the 1+1L PET pack @ mrp 2998 (= 2 x 1499 EL-1L master); the single 2L-can listing EDOGHZTJZEYQJGME also shows 2998 and zepto shows 2998 x34, while fresh/now/blinkit/bigbasket show master 2799 -&gt; mixed pack-variant pricing, flagged in master_mrp_stale with caveat.</t>
         </is>
       </c>
     </row>
@@ -8368,7 +8368,7 @@
       </c>
       <c r="M79" s="7" t="inlineStr">
         <is>
-          <t>identity verified (v2 CORRECT); prid owner-blessed from master sheet BLINKIT URL</t>
+          <t>identity verified (v2 CORRECT); prid owner-verified from master sheet BLINKIT URL</t>
         </is>
       </c>
     </row>
@@ -8920,7 +8920,7 @@
       </c>
       <c r="M89" s="7" t="inlineStr">
         <is>
-          <t>listing mrp 1799 vs master 1499 (owner-blessed pvid; live MRP differs)</t>
+          <t>listing mrp 1799 vs master 1499 (owner-verified pvid; live MRP differs)</t>
         </is>
       </c>
     </row>
@@ -9413,7 +9413,7 @@
       </c>
       <c r="M98" s="7" t="inlineStr">
         <is>
-          <t>blessed listing is the 1+1L pack; mrp 3598 = 2 x 1799 (the cross-platform-confirmed stale EV 1L mrp). Identity owner-blessed; see review for the master-vs-pack price basis question.</t>
+          <t>owner-verified listing is the 1+1L pack; mrp 3598 = 2 x 1799 (the cross-platform-confirmed stale EV 1L mrp). Identity owner-verified; see review for the master-vs-pack price basis question.</t>
         </is>
       </c>
     </row>
@@ -10318,7 +10318,7 @@
       </c>
       <c r="M115" s="7" t="inlineStr">
         <is>
-          <t>blessed pid mrp 350 vs master 225 (zepto shows 225 x75) -&gt; single-platform mrp_drift, see review.</t>
+          <t>owner-verified pid mrp 350 vs master 225 (zepto shows 225 x75) -&gt; single-platform mrp_drift, see review.</t>
         </is>
       </c>
     </row>
@@ -10923,7 +10923,7 @@
       </c>
       <c r="M126" s="7" t="inlineStr">
         <is>
-          <t>fk blessed mrp 560 == amazon/amazon-now/zepto 560 -&gt; ratifies LEAD-ruled master_mrp_stale (vs 400).</t>
+          <t>fk owner-verified mrp 560 == amazon/amazon-now/zepto 560 -&gt; ratifies LEAD-ruled master_mrp_stale (vs 400).</t>
         </is>
       </c>
     </row>
@@ -10982,7 +10982,7 @@
       </c>
       <c r="M127" s="7" t="inlineStr">
         <is>
-          <t>listing mrp modal 560 (1 store shows 400) vs master 400 (owner-blessed pvid; live MRP differs)</t>
+          <t>listing mrp modal 560 (1 store shows 400) vs master 400 (owner-verified pvid; live MRP differs)</t>
         </is>
       </c>
     </row>
@@ -11587,7 +11587,7 @@
       </c>
       <c r="M138" s="7" t="inlineStr">
         <is>
-          <t>identity verified (v2 CORRECT); prid owner-blessed from master sheet BLINKIT URL</t>
+          <t>identity verified (v2 CORRECT); prid owner-verified from master sheet BLINKIT URL</t>
         </is>
       </c>
     </row>
@@ -11864,7 +11864,7 @@
       </c>
       <c r="M143" s="7" t="inlineStr">
         <is>
-          <t>blessed pid is the 1+1L pack @ mrp 2098 (= 2 x 1049 POMACE-1L master); alt EDOGMHXYU2PHFW4N is the true 2L bottle @ 1449 == the LEAD-confirmed stale master mrp (amazon+bigbasket agree).</t>
+          <t>owner-verified pid is the 1+1L pack @ mrp 2098 (= 2 x 1049 POMACE-1L master); alt EDOGMHXYU2PHFW4N is the true 2L bottle @ 1449 == the LEAD-confirmed stale master mrp (amazon+bigbasket agree).</t>
         </is>
       </c>
     </row>
@@ -11923,7 +11923,7 @@
       </c>
       <c r="M144" s="7" t="inlineStr">
         <is>
-          <t>listing mrp 1449 vs master 1600 (owner-blessed pvid; live MRP differs)</t>
+          <t>listing mrp 1449 vs master 1600 (owner-verified pvid; live MRP differs)</t>
         </is>
       </c>
     </row>
@@ -12375,7 +12375,7 @@
       </c>
       <c r="M152" s="7" t="inlineStr">
         <is>
-          <t>identity verified (v2 CORRECT); prid owner-blessed from master sheet BLINKIT URL</t>
+          <t>identity verified (v2 CORRECT); prid owner-verified from master sheet BLINKIT URL</t>
         </is>
       </c>
     </row>
@@ -12846,7 +12846,7 @@
       </c>
       <c r="M161" s="7" t="inlineStr">
         <is>
-          <t>owner-blessed pid shows mrp 490 (sale 255) vs master 255; ALL other sources show 255 (zepto x60, blinkit x16, fresh x9, bigbasket, fk-minutes, fk dup QWRGDYBWXRTGFZFX). Single-listing mrp_drift on the blessed listing itself -&gt; see review.</t>
+          <t>owner-verified pid shows mrp 490 (sale 255) vs master 255; ALL other sources show 255 (zepto x60, blinkit x16, fresh x9, bigbasket, fk-minutes, fk dup QWRGDYBWXRTGFZFX). Single-listing mrp_drift on the owner-verified listing itself -&gt; see review.</t>
         </is>
       </c>
     </row>
@@ -13429,7 +13429,7 @@
       </c>
       <c r="M172" s="7" t="inlineStr">
         <is>
-          <t>blessed pid present in scrape but unpriced/OOS today (no mrp/sale).</t>
+          <t>owner-verified pid present in scrape but unpriced/OOS today (no mrp/sale).</t>
         </is>
       </c>
     </row>
@@ -14042,7 +14042,7 @@
       </c>
       <c r="M183" s="7" t="inlineStr">
         <is>
-          <t>blessed pid is the 1x3 (1+1+1L) pack @ mrp 2247 (= 3 x 749); amazon shows the same 2247 -&gt; in master_mrp_stale w/ caveat (amazon also lists 3050 = master).</t>
+          <t>owner-verified pid is the 1x3 (1+1+1L) pack @ mrp 2247 (= 3 x 749); amazon shows the same 2247 -&gt; in master_mrp_stale w/ caveat (amazon also lists 3050 = master).</t>
         </is>
       </c>
     </row>
@@ -14960,11 +14960,7 @@
           <t>https://www.amazon.in/dp/B0H2HDLB5Q?th=1</t>
         </is>
       </c>
-      <c r="E201" s="7" t="inlineStr">
-        <is>
-          <t>⚠ title not captured (listing not yet scraped)</t>
-        </is>
-      </c>
+      <c r="E201" s="7" t="inlineStr"/>
       <c r="F201" s="7" t="n"/>
       <c r="G201" s="7" t="n"/>
       <c r="H201" s="7" t="n"/>
@@ -14986,7 +14982,7 @@
       </c>
       <c r="M201" s="7" t="inlineStr">
         <is>
-          <t>identity from team master sheet v2 (2026-06-06); ASIN not in the 314-ASIN targeted scrape set yet (sheet says In Stock, seller Jivo Mart, url price 555)</t>
+          <t>identity from team master sheet v2 (2026-06-06); ASIN not in the 314-ASIN targeted scrape set yet (sheet says In Stock, seller Jivo Mart, url price 555); title not captured (listing not yet scraped)</t>
         </is>
       </c>
     </row>
@@ -16205,7 +16201,7 @@
       </c>
       <c r="M224" s="7" t="inlineStr">
         <is>
-          <t>fk blessed mrp 4599 == amazon sano-5L 4599 vs master 4499 -&gt; master_mrp_stale candidate (JIVO pomace 5L @4999 is a different SKU, widely live).</t>
+          <t>fk owner-verified mrp 4599 == amazon sano-5L 4599 vs master 4499 -&gt; master_mrp_stale candidate (JIVO pomace 5L @4999 is a different SKU, widely live).</t>
         </is>
       </c>
     </row>
@@ -16493,11 +16489,7 @@
           <t>https://www.amazon.in/dp/B0H2B92WLP?th=1</t>
         </is>
       </c>
-      <c r="E230" s="7" t="inlineStr">
-        <is>
-          <t>⚠ title not captured (listing not yet scraped)</t>
-        </is>
-      </c>
+      <c r="E230" s="7" t="inlineStr"/>
       <c r="F230" s="7" t="n"/>
       <c r="G230" s="7" t="n"/>
       <c r="H230" s="7" t="n"/>
@@ -16519,7 +16511,7 @@
       </c>
       <c r="M230" s="7" t="inlineStr">
         <is>
-          <t>identity from team master sheet v2 (2026-06-06); ASIN not in the 314-ASIN targeted scrape set yet (sheet says In Stock, seller Jivo Mart, url price 929)</t>
+          <t>identity from team master sheet v2 (2026-06-06); ASIN not in the 314-ASIN targeted scrape set yet (sheet says In Stock, seller Jivo Mart, url price 929); title not captured (listing not yet scraped)</t>
         </is>
       </c>
     </row>
@@ -16874,11 +16866,7 @@
           <t>https://www.amazon.in/dp/B0H2HJKJH1?th=1</t>
         </is>
       </c>
-      <c r="E237" s="7" t="inlineStr">
-        <is>
-          <t>⚠ title not captured (listing not yet scraped)</t>
-        </is>
-      </c>
+      <c r="E237" s="7" t="inlineStr"/>
       <c r="F237" s="7" t="n"/>
       <c r="G237" s="7" t="n"/>
       <c r="H237" s="7" t="n"/>
@@ -16900,7 +16888,7 @@
       </c>
       <c r="M237" s="7" t="inlineStr">
         <is>
-          <t>identity from team master sheet v2 (2026-06-06); ASIN not in the 314-ASIN targeted scrape set yet (sheet says Out of Stock)</t>
+          <t>identity from team master sheet v2 (2026-06-06); ASIN not in the 314-ASIN targeted scrape set yet (sheet says Out of Stock); title not captured (listing not yet scraped)</t>
         </is>
       </c>
     </row>
@@ -18357,7 +18345,7 @@
       </c>
       <c r="M264" s="7" t="inlineStr">
         <is>
-          <t>blessed pid is the 1L+1L+1L pack; mrp 825 == master exactly.</t>
+          <t>owner-verified pid is the 1L+1L+1L pack; mrp 825 == master exactly.</t>
         </is>
       </c>
     </row>
@@ -19511,11 +19499,7 @@
           <t>https://www.amazon.in/dp/B0GX19RGQH?th=1</t>
         </is>
       </c>
-      <c r="E286" s="7" t="inlineStr">
-        <is>
-          <t>⚠ title not captured (listing not yet scraped)</t>
-        </is>
-      </c>
+      <c r="E286" s="7" t="inlineStr"/>
       <c r="F286" s="7" t="n"/>
       <c r="G286" s="7" t="n"/>
       <c r="H286" s="7" t="n"/>
@@ -19537,7 +19521,7 @@
       </c>
       <c r="M286" s="7" t="inlineStr">
         <is>
-          <t>identity from team master sheet v2 (2026-06-06); ASIN not in the 314-ASIN targeted scrape set yet (sheet says Out of Stock)</t>
+          <t>identity from team master sheet v2 (2026-06-06); ASIN not in the 314-ASIN targeted scrape set yet (sheet says Out of Stock); title not captured (listing not yet scraped)</t>
         </is>
       </c>
     </row>
@@ -19899,7 +19883,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
     <col width="46" customWidth="1" min="3" max="3"/>
     <col width="46" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
@@ -20084,7 +20068,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>mrp 745 vs master 1049; LEAD-ruling cross-check: NO other platform shows 745 (1049 live on amazon-fresh x95, blinkit x152, zepto x55, amazon, bigbasket) -&gt; single-listing mrp_drift, review. Possibly a stale/seller-custom listing. Blessed pid EDOHYRPTDVEZVZ8E carries the mapping.</t>
+          <t>mrp 745 vs master 1049; LEAD-ruling cross-check: NO other platform shows 745 (1049 live on amazon-fresh x95, blinkit x152, zepto x55, amazon, bigbasket) -&gt; single-listing mrp_drift, review. Possibly a stale/seller-custom listing. owner-verified pid EDOHYRPTDVEZVZ8E carries the mapping.</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr"/>
@@ -20326,6 +20310,11 @@
           <t>flipkart</t>
         </is>
       </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>jivo-extra-light-3-litre-cooking-oil-olive-plastic-bottle</t>
+        </is>
+      </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
           <t>https://www.flipkart.com/jivo-extra-light-3-litre-cooking-oil-olive-plastic-bottle/p/itmf655d53b1f4f2</t>
@@ -20333,7 +20322,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>jivo-extra-light-3-litre-cooking-oil-olive-plastic-bottle (owner sheet URL)</t>
+          <t>Jivo Extra Light Olive Oil - 3 Litre | Imported from Spain | Recommended for Daily Cooking – Roasting, Frying, Baking &amp; All Types of Cuisines | Low in Saturated Fat</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -20343,7 +20332,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>owner sheet has a FLIPKART URL for EXTRA LIGHT 3L but it carries NO pid (cannot resolve offline, network calls forbidden). Two scraped 1+1+1L listings have 3L-style names: EDOHYRPCTWGRKWKU 'JIVO Extra Light Cooking 3 Liter ... Plastic Bottle' (unpriced) and QWRGEMPJJGDRYACC 'Jivo Extra Light Daily Cooking Olive Oil 3 Litre ...' (mrp 2475, sale 1647, sap FG0000310); master mrp 2200 matches neither (third sibling EDOGE5WYGYXCRRMF @4497=3x1499). Mapping left null; the 3 listings stay in unpriced. Needs the pid from the live URL.</t>
+          <t>owner sheet has a FLIPKART URL for EXTRA LIGHT 3L but it carries NO pid (cannot resolve offline, network calls forbidden). Two scraped 1+1+1L listings have 3L-style names: EDOHYRPCTWGRKWKU 'JIVO Extra Light Cooking 3 Liter ... Plastic Bottle' (unpriced) and QWRGEMPJJGDRYACC 'Jivo Extra Light Daily Cooking Olive Oil 3 Litre ...' (mrp 2475, sale 1647, sap FG0000310); master mrp 2200 matches neither (third sibling EDOGE5WYGYXCRRMF @4497=3x1499). Mapping left null; the 3 listings stay in unpriced. Needs the pid from the live URL.; title annotation moved: (owner sheet URL); url-slug (not a title): jivo-extra-light-3-litre-cooking-oil-olive-plastic-bottle; title from e-com master sheet (listing not resolvable offline)</t>
         </is>
       </c>
       <c r="G14" s="9" t="inlineStr"/>
@@ -20376,7 +20365,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>owner-blessed pid (mapping KEPT) but mrp 490 vs master/everywhere-else 255 (sale 255 == master mrp!). Single-listing drift per LEAD ruling. Dup QWRGDYBWXRTGFZFX shows the clean 255/217 and is kept as alt — consider re-blessing it.</t>
+          <t>owner-verified pid (mapping KEPT) but mrp 490 vs master/everywhere-else 255 (sale 255 == master mrp!). Single-listing drift per LEAD ruling. Dup QWRGDYBWXRTGFZFX shows the clean 255/217 and is kept as alt — consider re-blessing it.</t>
         </is>
       </c>
       <c r="G15" s="9" t="inlineStr"/>
@@ -20409,7 +20398,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>mapping KEPT (owner-blessed); mrp 350 vs master 225, zepto shows 225 x75 -&gt; flipkart-only mrp_drift per LEAD ruling.</t>
+          <t>mapping KEPT (owner-verified); mrp 350 vs master 225, zepto shows 225 x75 -&gt; flipkart-only mrp_drift per LEAD ruling.</t>
         </is>
       </c>
       <c r="G16" s="9" t="inlineStr"/>
@@ -20475,7 +20464,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>mapping KEPT (owner-blessed) but the pid is a 1+1L pack @ mrp 3598 = 2x1799 (stale EV-1L mrp), not a single 2L bottle (master 2700; amazon lists a 2998 EV-2L, W4 flagged separately). Price-match comparisons for EV 2L on flipkart will be on pack arithmetic, not the 2L bottle.</t>
+          <t>mapping KEPT (owner-verified) but the pid is a 1+1L pack @ mrp 3598 = 2x1799 (stale EV-1L mrp), not a single 2L bottle (master 2700; amazon lists a 2998 EV-2L, W4 flagged separately). Price-match comparisons for EV 2L on flipkart will be on pack arithmetic, not the 2L bottle.</t>
         </is>
       </c>
       <c r="G18" s="9" t="inlineStr"/>
@@ -20548,11 +20537,7 @@
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>⚠ title not captured (listing not yet scraped)</t>
-        </is>
-      </c>
+      <c r="D21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>APPLIED verify_results corrections to the BB fragment: (1) 'Fizzy Water Flavoured With Lemon' 40335332 remapped SPRING WATER 750ML -&gt; SODA LEMON 750ML (URL slug 'fizzy-water-lemon-flavoured-carbonated-water' + mrp 55 = master 55 confirm); (2) 'Canola Omega-3 Rich Cooking Oil 1 L' 40309979 remapped CANOLA 1L -&gt; CANOLA 1L POUCH (URL slug ends '...-1-l-pouch' + mrp 299 = pouch master 299 confirm). Both marked method=VERIFY-CORRECTED+MRP, confidence=anchored.</t>
@@ -20562,11 +20547,7 @@
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>⚠ title not captured (listing not yet scraped)</t>
-        </is>
-      </c>
+      <c r="D22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>LEAD RULING APPLIED (bus.md): BB EXTRA VIRGIN 1L (1799) and JIVO POMACE 2L (1449) divergences are multi-platform confirmed (W1 amazon-family + W3 zepto show identical MRPs) -&gt; moved from mrp_drift to the new master_mrp_stale section; mapping confidence set to 'anchored' with identity-certain note (was anchored-with-mrp-drift per the original task spec — ruling supersedes). mrp_drift now holds only single-platform divergences (amazon EXTRA LIGHT 3L 2997v2200, EXTRA VIRGIN 2L 2998v2700 — W1 should confirm or fold).</t>
@@ -20576,11 +20557,7 @@
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>⚠ title not captured (listing not yet scraped)</t>
-        </is>
-      </c>
+      <c r="D23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>BB run is a single national 'All India' member-price session (1 pincode), so sale_modal=sale_min=sale_max for every row; prices are MEMBER prices (logged-in cookie session), not guest prices.</t>
@@ -20590,11 +20567,7 @@
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>⚠ title not captured (listing not yet scraped)</t>
-        </is>
-      </c>
+      <c r="D24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>BB coverage: 14 of 96 master products present on bigbasket; 82 mapped null. 9 BB listings are NOT-IN-MASTER (7x wheatgrass 200ml, 1x wheatgrass 500ml mango, 1x Indian Tonic Water 200ml) — all folded into the census.</t>
@@ -20604,11 +20577,7 @@
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>⚠ title not captured (listing not yet scraped)</t>
-        </is>
-      </c>
+      <c r="D25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>CENSUS REFINEMENTS vs verify_results 'gaps' first pass: (a) amazon-now removed from WHEATGRASS 200ML platforms (its only unmatched listing is the 500ml mango); (b) SANO CANOLA 2L split out of CANOLA 2L (sister brand); (c) added DESI GHEE 500G/1KG families (live mis-matches to A2 GHEE, invisible to gaps because they sat in auto_matches, not not_in_master); (d) added SANO POMACE 3L (WRONG-matched to SANO POMACE 1L) and SANO POMACE 2L (missed); (e) added 4th amazon gift hamper B0FQC831P8; (f) PUNJABI JEERA 160 ML 24 PCS (flipkart ARDHCJMTXHZ5HQDA) is NOT a gap — master 'PUNJABI JEERA 160ML' IS the Pack-of-24 SKU (mrp 240); it's a name-heuristic miss like SANO_CLASSIC 5L and Coffee 100g.</t>
@@ -20618,11 +20587,7 @@
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>⚠ title not captured (listing not yet scraped)</t>
-        </is>
-      </c>
+      <c r="D26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>Name-heuristic misses (exist in master, scraper failed to match — fix the matcher, do not add SKUs): SANO_CLASSIC 5L flipkart EDOHAGDYVQWT6GNG (underscore), Coffee 100g flipkart CFEGMJ5GJE7HD3DQ (mrp 350 = master COFFEE exactly), PUNJABI JEERA 160 ML 24 PCS flipkart ARDHCJMTXHZ5HQDA (master row is itself a pack-of-24).</t>
@@ -20632,11 +20597,7 @@
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>⚠ title not captured (listing not yet scraped)</t>
-        </is>
-      </c>
+      <c r="D27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>DISAGREE with gaps on amazon COCONUT 1L B0D6NFLL3M (vol 2000, mrp 1400): gaps called vol a scraper bug + a Rs.700 MRP discrepancy; evidence says it is a 1L x2 twin-pack — mrp is exactly 2x master (700) and sibling ASIN B0CZP2HPGL has identical vol/mrp with an explicit '(Pack of' marker. Treated as combo, not drift.</t>
@@ -20646,11 +20607,7 @@
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>⚠ title not captured (listing not yet scraped)</t>
-        </is>
-      </c>
+      <c r="D28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>AMBIGUOUS (needs PDP check, not asserted): amazon EXTRA VIRGIN 200ML B0GG7QM7LY (vol 400 suggests a 2-pack but mrp 598 != 2x350=700); amazon-fresh mustard B0GZZS8J7Q (title 1L, vol 2000, mrp 540 — 2L bottle or 1Lx2 pack at 540?); amazon MUSTARD 2L B0CGZQMJHY mrp 3750 (likely data error, ~7x the 1L price).</t>
@@ -20660,11 +20617,7 @@
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>⚠ title not captured (listing not yet scraped)</t>
-        </is>
-      </c>
+      <c r="D29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>amazon B0BGPGRP4Z ('Mustard 5L &amp;JIVO...' vol 6000 mrp 1505 = 1250+255 exactly) reclassified as a 5L+1L combo despite combo=false flag; the combo flag in the raw data under-counts amazon 'X &amp; Y (Pack of 2)' bundles broadly.</t>
@@ -20674,11 +20627,7 @@
     </row>
     <row r="30">
       <c r="A30" t="inlineStr"/>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>⚠ title not captured (listing not yet scraped)</t>
-        </is>
-      </c>
+      <c r="D30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>Combos/multipacks EXCLUDED from the census: 277 deduplicated bundle/multipack listings (incl. flipkart WG 3/6-packs, TEA pack-of-2/3/4, SOYABEAN 1L 3PCS EDOGGP4FSQVM2ERR, and ~50 amazon 'X &amp; Y each' two-product bundles mis-flagged combo=false). gaps' combo_count of 169 used a different dedupe. Suggest a dedicated combo sheet priced from component master rows.</t>
@@ -20688,11 +20637,7 @@
     </row>
     <row r="31">
       <c r="A31" t="inlineStr"/>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>⚠ title not captured (listing not yet scraped)</t>
-        </is>
-      </c>
+      <c r="D31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
           <t>amazon also sells a WHEATGRASS 250ML flavour line (cola B09MJ3KLFP, jeera B0C1V6DG9C, lemon B09TWL9RFR, orange B09MHZLRSG) — only as multipacks, so left in the combos bucket; flag to e-comm team as an unpriced single-unit line if single packs appear.</t>
@@ -20702,11 +20647,7 @@
     </row>
     <row r="32">
       <c r="A32" t="inlineStr"/>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>⚠ title not captured (listing not yet scraped)</t>
-        </is>
-      </c>
+      <c r="D32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
           <t>mrp_drift includes 2 amazon rows (EXTRA LIGHT 3L 2997 vs 2200, EXTRA VIRGIN 2L 2998 vs 2700) surfaced by the cross-platform census sweep; the amazon master-map fragment itself is W1's scope — dedupe on merge if W1 reports the same.</t>
@@ -20716,11 +20657,7 @@
     </row>
     <row r="33">
       <c r="A33" t="inlineStr"/>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>⚠ title not captured (listing not yet scraped)</t>
-        </is>
-      </c>
+      <c r="D33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
           <t>No W1/W2/W3 unpriced findings were on bus.md at finalize time; census built from dryrun.json + verify_input.json + verify_results.json only.</t>
@@ -21119,7 +21056,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>FYI, mapping NOT changed: EXTRA VIRGIN 2L's owner-blessed flipkart slot is itself a 1+1L pack (mrp 3598 = 2x stale 1799). Now that a true EXTRA VIRGIN 1L + 1L master row exists (mapped to QWRGEMNS9ZPZGWJH @2998), owner may want to re-point the EV 2L slot</t>
+          <t>FYI, mapping NOT changed: EXTRA VIRGIN 2L's owner-verified flipkart slot is itself a 1+1L pack (mrp 3598 = 2x stale 1799). Now that a true EXTRA VIRGIN 1L + 1L master row exists (mapped to QWRGEMNS9ZPZGWJH @2998), owner may want to re-point the EV 2L slot</t>
         </is>
       </c>
       <c r="G45" s="9" t="inlineStr"/>
@@ -21265,7 +21202,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>flipkart 398 on BOTH listings (blessed EDOHF5F6BS3MEHJD + EDOGWGZGCC8YG5PZ); amazon 399 + amazon-fresh 399 (Re.1 rounding, same convention as W3 GOLD 5L re-verdict). LEAD asked W2 to cross-check this exact case -&gt; stale, mapping kept.</t>
+          <t>flipkart 398 on BOTH listings (owner-verified EDOHF5F6BS3MEHJD + EDOGWGZGCC8YG5PZ); amazon 399 + amazon-fresh 399 (Re.1 rounding, same convention as W3 GOLD 5L re-verdict). LEAD asked W2 to cross-check this exact case -&gt; stale, mapping kept.</t>
         </is>
       </c>
     </row>
@@ -21293,7 +21230,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>flipkart 1799 on both listings RATIFIES the already-ruled stale (amazon-fresh/now). | [{'platform': 'bigbasket', 'listing': 'Extra Virgin Olive Oil - Antioxidants Rich, Suitable For Salads, Saute', 'id': '40250808', 'mrp': 1799}, {'platform': 'zepto', 'listing': 'per W3 owner-blessed pvid', 'mrp': 1799}, {'platform': 'amazon-fresh/amazon-now', 'listing': 'per W1 cross-check', 'mrp': 1799}]</t>
+          <t>flipkart 1799 on both listings RATIFIES the already-ruled stale (amazon-fresh/now). | [{'platform': 'bigbasket', 'listing': 'Extra Virgin Olive Oil - Antioxidants Rich, Suitable For Salads, Saute', 'id': '40250808', 'mrp': 1799}, {'platform': 'zepto', 'listing': 'per W3 owner-verified pvid', 'mrp': 1799}, {'platform': 'amazon-fresh/amazon-now', 'listing': 'per W1 cross-check', 'mrp': 1799}]</t>
         </is>
       </c>
     </row>
@@ -21321,7 +21258,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>flipkart blessed 560 RATIFIES the already-ruled stale (amazon, amazon-now, zepto x51). | [{'platform': 'zepto', 'listing': 'per W3 owner-blessed pvid', 'mrp': 560}, {'platform': 'amazon-now', 'listing': 'per W1 cross-check', 'mrp': 560}]</t>
+          <t>flipkart owner-verified 560 RATIFIES the already-ruled stale (amazon, amazon-now, zepto x51). | [{'platform': 'zepto', 'listing': 'per W3 owner-verified pvid', 'mrp': 560}, {'platform': 'amazon-now', 'listing': 'per W1 cross-check', 'mrp': 560}]</t>
         </is>
       </c>
     </row>
@@ -21349,7 +21286,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>flipkart 2L-bottle alt EDOGMHXYU2PHFW4N @1449 RATIFIES the already-ruled stale (amazon, bigbasket). | [{'platform': 'bigbasket', 'listing': 'Pomace Olive Oil 2L', 'id': '40309980', 'mrp': 1449}, {'platform': 'zepto', 'listing': 'per W3 owner-blessed pvid', 'mrp': 1449}, {'platform': 'amazon', 'listing': 'per W1 cross-check', 'mrp': 1449}]</t>
+          <t>flipkart 2L-bottle alt EDOGMHXYU2PHFW4N @1449 RATIFIES the already-ruled stale (amazon, bigbasket). | [{'platform': 'bigbasket', 'listing': 'Pomace Olive Oil 2L', 'id': '40309980', 'mrp': 1449}, {'platform': 'zepto', 'listing': 'per W3 owner-verified pvid', 'mrp': 1449}, {'platform': 'amazon', 'listing': 'per W1 cross-check', 'mrp': 1449}]</t>
         </is>
       </c>
     </row>
@@ -21377,7 +21314,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>flipkart 4599 (blessed) + amazon sano-pomace-5L 4599. (4999 elsewhere is JIVO pomace 5L, a different SKU.) 2 platforms -&gt; stale.</t>
+          <t>flipkart 4599 (owner-verified) + amazon sano-pomace-5L 4599. (4999 elsewhere is JIVO pomace 5L, a different SKU.) 2 platforms -&gt; stale.</t>
         </is>
       </c>
     </row>
@@ -28099,7 +28036,7 @@
         <v>540</v>
       </c>
       <c r="E230" s="7" t="inlineStr"/>
-      <c r="F230" s="7" t="n"/>
+      <c r="F230" s="7" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" s="8" t="inlineStr">
@@ -29806,7 +29743,7 @@
     <row r="290">
       <c r="A290" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">    SUNFLOWER OIL 2L ⚠ internal name (listing not yet scraped)</t>
+          <t xml:space="preserve">    (title not captured)</t>
         </is>
       </c>
       <c r="B290" s="7" t="inlineStr">
@@ -29823,7 +29760,7 @@
       <c r="E290" s="7" t="inlineStr"/>
       <c r="F290" s="7" t="inlineStr">
         <is>
-          <t>SUNFLOWER OIL 2L</t>
+          <t>internal name: SUNFLOWER OIL 2L — listing not yet scraped, no on-page title</t>
         </is>
       </c>
     </row>
@@ -29910,7 +29847,7 @@
     <row r="294">
       <c r="A294" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">    CANOLA 5L + MUSTARD 5L + SUNFLOWER 5L ⚠ internal name (listing not yet scraped)</t>
+          <t xml:space="preserve">    (title not captured)</t>
         </is>
       </c>
       <c r="B294" s="7" t="inlineStr">
@@ -29931,7 +29868,7 @@
       </c>
       <c r="F294" s="7" t="inlineStr">
         <is>
-          <t>CANOLA 5L + MUSTARD 5L + SUNFLOWER 5L</t>
+          <t>internal name: CANOLA 5L + MUSTARD 5L + SUNFLOWER 5L — listing not yet scraped, no on-page title</t>
         </is>
       </c>
     </row>
@@ -30126,7 +30063,7 @@
     <row r="302">
       <c r="A302" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">    MUSTARD 5L + SUNFLOWER 5L ⚠ internal name (listing not yet scraped)</t>
+          <t xml:space="preserve">    (title not captured)</t>
         </is>
       </c>
       <c r="B302" s="7" t="inlineStr">
@@ -30147,7 +30084,7 @@
       </c>
       <c r="F302" s="7" t="inlineStr">
         <is>
-          <t>MUSTARD 5L + SUNFLOWER 5L</t>
+          <t>internal name: MUSTARD 5L + SUNFLOWER 5L — listing not yet scraped, no on-page title</t>
         </is>
       </c>
     </row>
@@ -30870,7 +30807,7 @@
     <row r="328">
       <c r="A328" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">    CANOLA 1L + SOYABEAN 1L + SUNFLOWER 1L ⚠ internal name (listing not yet scraped)</t>
+          <t xml:space="preserve">    (title not captured)</t>
         </is>
       </c>
       <c r="B328" s="7" t="inlineStr">
@@ -30891,7 +30828,7 @@
       </c>
       <c r="F328" s="7" t="inlineStr">
         <is>
-          <t>CANOLA 1L + SOYABEAN 1L + SUNFLOWER 1L</t>
+          <t>internal name: CANOLA 1L + SOYABEAN 1L + SUNFLOWER 1L — listing not yet scraped, no on-page title</t>
         </is>
       </c>
     </row>
@@ -31272,7 +31209,7 @@
     <row r="342">
       <c r="A342" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">    EXTRA VIRGIN 5L + EXTRA LIGHT 5L + JIVO POMACE 5L ⚠ internal name (listing not yet scraped)</t>
+          <t xml:space="preserve">    (title not captured)</t>
         </is>
       </c>
       <c r="B342" s="7" t="inlineStr">
@@ -31293,7 +31230,7 @@
       </c>
       <c r="F342" s="7" t="inlineStr">
         <is>
-          <t>EXTRA VIRGIN 5L + EXTRA LIGHT 5L + JIVO POMACE 5L</t>
+          <t>internal name: EXTRA VIRGIN 5L + EXTRA LIGHT 5L + JIVO POMACE 5L — listing not yet scraped, no on-page title</t>
         </is>
       </c>
     </row>

</xml_diff>